<commit_message>
Hiring workbook: add Other open roles tab and conflict C5
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016P9Z9B879NzE7WcSVWNcxZ
</commit_message>
<xml_diff>
--- a/Analysis/output/Sales_hiring_raw_data.xlsx
+++ b/Analysis/output/Sales_hiring_raw_data.xlsx
@@ -10,9 +10,10 @@
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Timeline (raw)" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Roster reqs (raw)" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Conflicts" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Open actions" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Other open roles" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Roster reqs (raw)" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Conflicts" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Open actions" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -255,6 +256,64 @@
     <author>Unknown Author</author>
   </authors>
   <commentList>
+    <comment ref="A3" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Raj: Eng has 'a couple open but no urgency' (slack L217), but the roster lists only one Eng req.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">In the roster but missing from Elena's May 1 'official picture' (slack L222).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A5" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">No target start date (roster L25), so urgency can't be judged. Also missing from Elena's May 1 list (slack L222).</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A6" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Not in the roster at all. Sofia: 'one backfill open' (L214); confirmed unaffected by the freeze and proceeding (L236, L239).</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <authors>
+    <author>Unknown Author</author>
+  </authors>
+  <commentList>
     <comment ref="B9" authorId="0">
       <text>
         <r>
@@ -272,7 +331,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="290" uniqueCount="188">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="264">
   <si>
     <t xml:space="preserve">Q2 — Sales hiring: hire or freeze? Current state and owner</t>
   </si>
@@ -358,6 +417,15 @@
     <t xml:space="preserve">4 independent sources agree (Dana, Priya, Elena, minutes); no later reversal.</t>
   </si>
   <si>
+    <t xml:space="preserve">Other teams' open roles</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unaffected — see 'Other open roles'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4 open non-Sales roles (roster and People's list disagree — Conflict C5); 2 more proposed for Q3.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Confidence — follow-through</t>
   </si>
   <si>
@@ -625,6 +693,216 @@
     <t xml:space="preserve">Q3 planning: don't submit Sales reqs while the freeze holds. Latest statement in the bundle; still frozen.</t>
   </si>
   <si>
+    <t xml:space="preserve">Non-Sales roles. The freeze is Sales-only ('Other teams' open reqs are unaffected' — slack L79, L236), so these stay open. Roster and People's list don't agree — see Flag and Conflict C5.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Req ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Team</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hiring manager</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Target start</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affected by Sales freeze?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In roster (May 1)?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In People's May 1 list?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raw source (verbatim)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backend Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-118</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raj Patel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-08-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (L23)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes — 'an Eng role' (slack L222)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-118,Engineering,Backend Engineer,OPEN,2026-08-01,Raj Patel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">headcount_roster.csv:L23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CHECK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Raj: Eng has 'a couple open but no urgency' (slack L217), but the roster lists only one Eng req.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Senior Video Editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-121</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Content/Production</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yuki Tanaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-07-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (L24)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-121,Content/Production,Senior Video Editor,OPEN,2026-07-01,Yuki Tanaka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">headcount_roster.csv:L24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CONFLICT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In the roster but missing from Elena's May 1 'official picture' (slack L222).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analytics Engineer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-125</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Okoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— (blank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (L25)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REQ-125,Data,Analytics Engineer,OPEN,,Ben Okoro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">headcount_roster.csv:L25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No target start date (roster L25), so urgency can't be judged. Also missing from Elena's May 1 list (slack L222).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creator Management backfill</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— (no req ID)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Creator Management</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open — proceeding</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes (slack L222)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfect, proceeding with the backfill then.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slack_export.md:L239</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in the roster at all. Sofia: 'one backfill open' (L214); confirmed unaffected by the freeze and proceeding (L236, L239).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lifecycle marketer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">— (proposed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth/Marketing</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hannah Cole</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposed for Q3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth might want a lifecycle marketer. Will write it up.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slack_export.md:L247</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROPOSED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not a req yet. Hannah 'will write it up' for Q3 planning; requests due end of June (slack L243).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post-production video editor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Post production could use another editor — that's the real bottleneck, not shooting. Will submit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slack_export.md:L250</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yuki 'will submit'; post is the real bottleneck (also L34). Unclear if additional to REQ-121 or overlapping.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open non-Sales roles (roster + People list, excl. proposed)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…of which in the roster</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…of which in People's May 1 list</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proposed for Q3 (not yet reqs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affected by the Sales freeze</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bounds: 4 open non-Sales roles in the union of both sources; 5+ if Engineering really has 'a couple' open (slack L217). Unblock with a Greenhouse export or an updated req list from Elena.</t>
+  </si>
+  <si>
     <t xml:space="preserve">headcount_roster.csv — header and OPEN_REQUISITIONS section, verbatim (lines 1–4, 20–25).</t>
   </si>
   <si>
@@ -649,18 +927,9 @@
     <t xml:space="preserve">REQ-114 APPROVED as of 2026-05-01. Frozen/paused since 2026-06-10: slack L67 (Dana), L70 (Priya), L230 (Elena: 'May 1 roster is now stale'), leadership_sync L16 ('superseded by this decision').</t>
   </si>
   <si>
-    <t xml:space="preserve">REQ-118,Engineering,Backend Engineer,OPEN,2026-08-01,Raj Patel</t>
-  </si>
-  <si>
     <t xml:space="preserve">Not Sales; freeze is Sales-only (slack L79, L236), so unaffected.</t>
   </si>
   <si>
-    <t xml:space="preserve">REQ-121,Content/Production,Senior Video Editor,OPEN,2026-07-01,Yuki Tanaka</t>
-  </si>
-  <si>
-    <t xml:space="preserve">REQ-125,Data,Analytics Engineer,OPEN,,Ben Okoro</t>
-  </si>
-  <si>
     <t xml:space="preserve">Also not in the roster: the Creator Management backfill Elena mentions on May 1 (slack L222). The roster isn't the full req picture.</t>
   </si>
   <si>
@@ -775,10 +1044,28 @@
     <t xml:space="preserve">Confirm with Priya</t>
   </si>
   <si>
+    <t xml:space="preserve">C5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which non-Sales roles are open?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">headcount_roster.csv L23–L25 — REQ-118 (Eng), REQ-121 (Content), REQ-125 (Data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">slack L222 (Elena, May 1, 'official picture') — Sales AE, Creator Mgmt backfill, one Eng role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neither list is complete. Union = 4 open non-Sales roles (5+ if Eng has 'a couple', L217).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open-role count 4–5+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greenhouse export / updated req list (Elena)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Follow-ups assigned with the decision. Status is what the bundle shows, not what probably happened.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
   </si>
   <si>
     <t xml:space="preserve">Action (verbatim from minutes)</t>
@@ -992,7 +1279,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1062,6 +1349,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1325,7 +1616,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -1472,21 +1763,32 @@
       <c r="A15" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="4" t="s">
+      <c r="B15" s="3" t="s">
         <v>29</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>31</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1523,42 +1825,42 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1569,27 +1871,27 @@
         <v>46133.3965277778</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D3" s="8" t="n">
         <v>17</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I3" s="8"/>
       <c r="J3" s="8"/>
       <c r="K3" s="8" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1600,27 +1902,27 @@
         <v>46133.4027777778</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D4" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I4" s="8"/>
       <c r="J4" s="8"/>
       <c r="K4" s="8" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1631,27 +1933,27 @@
         <v>46133.4055555556</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>23</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I5" s="8"/>
       <c r="J5" s="8"/>
       <c r="K5" s="8" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1662,27 +1964,27 @@
         <v>46133.4111111111</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D6" s="8" t="n">
         <v>26</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I6" s="8"/>
       <c r="J6" s="8"/>
       <c r="K6" s="8" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1693,27 +1995,27 @@
         <v>46143</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D7" s="8" t="n">
         <v>2</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I7" s="8"/>
       <c r="J7" s="11"/>
       <c r="K7" s="8" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,29 +2026,29 @@
         <v>46143</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D8" s="8" t="n">
         <v>22</v>
       </c>
       <c r="E8" s="8" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G8" s="12" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I8" s="8"/>
       <c r="J8" s="13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K8" s="8" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1757,29 +2059,29 @@
         <v>46143.6875</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D9" s="8" t="n">
         <v>222</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G9" s="12" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H9" s="12" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I9" s="8"/>
       <c r="J9" s="13" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="K9" s="8" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1790,27 +2092,27 @@
         <v>46143.6951388889</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D10" s="8" t="n">
         <v>225</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G10" s="8" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H10" s="8" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I10" s="8"/>
       <c r="J10" s="8"/>
       <c r="K10" s="8" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1821,31 +2123,31 @@
         <v>46183.3659722222</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D11" s="8" t="n">
         <v>67</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G11" s="14" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I11" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J11" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K11" s="8" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1856,27 +2158,27 @@
         <v>46183.3694444444</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D12" s="8" t="n">
         <v>70</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H12" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
       <c r="K12" s="8" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1887,27 +2189,27 @@
         <v>46183.3784722222</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D13" s="8" t="n">
         <v>73</v>
       </c>
       <c r="E13" s="8" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="F13" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G13" s="8" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H13" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
       <c r="K13" s="8" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1918,27 +2220,27 @@
         <v>46183.3826388889</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D14" s="8" t="n">
         <v>76</v>
       </c>
       <c r="E14" s="8" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="F14" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G14" s="8" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="H14" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I14" s="8"/>
       <c r="J14" s="8"/>
       <c r="K14" s="8" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1949,31 +2251,31 @@
         <v>46183.3847222222</v>
       </c>
       <c r="C15" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>79</v>
       </c>
       <c r="E15" s="8" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="F15" s="8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="G15" s="14" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J15" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K15" s="8" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1984,27 +2286,27 @@
         <v>46184</v>
       </c>
       <c r="C16" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D16" s="8" t="n">
         <v>15</v>
       </c>
       <c r="E16" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G16" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H16" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I16" s="8"/>
       <c r="J16" s="11"/>
       <c r="K16" s="8" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2015,31 +2317,31 @@
         <v>46184</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D17" s="8" t="n">
         <v>16</v>
       </c>
       <c r="E17" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G17" s="14" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J17" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K17" s="8" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2050,29 +2352,29 @@
         <v>46184</v>
       </c>
       <c r="C18" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D18" s="8" t="n">
         <v>17</v>
       </c>
       <c r="E18" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G18" s="16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H18" s="16" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I18" s="8"/>
       <c r="J18" s="17" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="K18" s="8" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,31 +2385,31 @@
         <v>46184</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D19" s="8" t="n">
         <v>18</v>
       </c>
       <c r="E19" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="J19" s="15" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="K19" s="8" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2118,27 +2420,27 @@
         <v>46184</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D20" s="8" t="n">
         <v>19</v>
       </c>
       <c r="E20" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I20" s="8"/>
       <c r="J20" s="8"/>
       <c r="K20" s="8" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2149,29 +2451,29 @@
         <v>46184</v>
       </c>
       <c r="C21" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D21" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E21" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H21" s="16" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I21" s="8"/>
       <c r="J21" s="17" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2182,29 +2484,29 @@
         <v>46184</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D22" s="8" t="n">
         <v>21</v>
       </c>
       <c r="E22" s="8" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="G22" s="16" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H22" s="16" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I22" s="8"/>
       <c r="J22" s="17" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2215,27 +2517,27 @@
         <v>46184.3958333333</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D23" s="8" t="n">
         <v>230</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I23" s="8"/>
       <c r="J23" s="8"/>
       <c r="K23" s="8" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2246,27 +2548,27 @@
         <v>46184.4013888889</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D24" s="8" t="n">
         <v>233</v>
       </c>
       <c r="E24" s="8" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G24" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="H24" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="I24" s="8"/>
       <c r="J24" s="11"/>
       <c r="K24" s="8" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2277,27 +2579,27 @@
         <v>46184.4034722222</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D25" s="8" t="n">
         <v>236</v>
       </c>
       <c r="E25" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I25" s="8"/>
       <c r="J25" s="8"/>
       <c r="K25" s="8" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2308,27 +2610,27 @@
         <v>46188.5833333333</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>244</v>
       </c>
       <c r="E26" s="8" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H26" s="8" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="I26" s="8"/>
       <c r="J26" s="8"/>
       <c r="K26" s="8" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
   </sheetData>
@@ -2348,132 +2650,364 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="80"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="60"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>37</v>
+        <v>121</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>43</v>
+        <v>123</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="n">
+        <v>124</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="G2" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="H2" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="I2" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="J2" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="K2" s="7" t="s">
+        <v>131</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>132</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>135</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>136</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>138</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="J3" s="8" t="s">
+        <v>140</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>141</v>
+      </c>
+      <c r="L3" s="17" t="s">
+        <v>142</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>149</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J4" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="K4" s="8" t="s">
+        <v>151</v>
+      </c>
+      <c r="L4" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="M4" s="8" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>155</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>156</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="F5" s="16" t="s">
+        <v>158</v>
+      </c>
+      <c r="G5" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H5" s="8" t="s">
+        <v>159</v>
+      </c>
+      <c r="I5" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J5" s="8" t="s">
+        <v>160</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>161</v>
+      </c>
+      <c r="L5" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>163</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>164</v>
+      </c>
+      <c r="C6" s="8" t="s">
+        <v>165</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>113</v>
+      </c>
+      <c r="E6" s="8" t="s">
+        <v>166</v>
+      </c>
+      <c r="F6" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G6" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>167</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>168</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>169</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>173</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>174</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>176</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>177</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>172</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>175</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>158</v>
+      </c>
+      <c r="G8" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>182</v>
+      </c>
+      <c r="L8" s="18" t="s">
+        <v>178</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B10" s="4" t="n">
+        <f aca="false">COUNTIFS($E$3:$E$8,"OPEN")+COUNTIFS($E$3:$E$8,"Open*proceeding")</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" s="4" t="n">
+        <f aca="false">COUNTIFS($H$3:$H$8,"Yes*")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" s="4" t="n">
+        <f aca="false">COUNTIFS($I$3:$I$8,"Yes*")</f>
         <v>2</v>
       </c>
-      <c r="B4" s="5" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="C9" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="n">
-        <v>23</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>126</v>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" s="4" t="n">
+        <f aca="false">COUNTIFS($E$3:$E$8,"Proposed*")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>129</v>
+      <c r="A14" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="B14" s="4" t="n">
+        <f aca="false">COUNTIFS($G$3:$G$8,"Yes")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -2493,7 +3027,152 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:D14"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="80"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="4" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>191</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" s="5" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B9" s="19" t="s">
+        <v>69</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="2" t="s">
+        <v>199</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <legacyDrawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2508,137 +3187,163 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>130</v>
+        <v>200</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>131</v>
+        <v>201</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>132</v>
+        <v>202</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>133</v>
+        <v>203</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>134</v>
+        <v>204</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>135</v>
+        <v>205</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>136</v>
+        <v>206</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>137</v>
+        <v>207</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>138</v>
+        <v>208</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>139</v>
+        <v>209</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>141</v>
+        <v>211</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>142</v>
+        <v>212</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>143</v>
+        <v>213</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>144</v>
+        <v>214</v>
       </c>
       <c r="G3" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H3" s="8" t="s">
-        <v>145</v>
+        <v>215</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>146</v>
+        <v>216</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>147</v>
+        <v>217</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>148</v>
+        <v>218</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>149</v>
+        <v>219</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>150</v>
+        <v>220</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>151</v>
+        <v>221</v>
       </c>
       <c r="G4" s="8" t="s">
         <v>26</v>
       </c>
       <c r="H4" s="8" t="s">
-        <v>152</v>
+        <v>222</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>153</v>
+        <v>223</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>154</v>
+        <v>224</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>155</v>
+        <v>225</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>156</v>
+        <v>226</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>157</v>
+        <v>227</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>158</v>
+        <v>228</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H5" s="8" t="s">
-        <v>159</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>160</v>
+        <v>230</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>161</v>
+        <v>231</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>162</v>
+        <v>232</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>163</v>
+        <v>233</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>164</v>
+        <v>234</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>165</v>
+        <v>235</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="H6" s="8" t="s">
-        <v>166</v>
+        <v>236</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="B7" s="8" t="s">
+        <v>238</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>240</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -2652,7 +3357,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -2671,99 +3376,99 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="4" t="s">
-        <v>167</v>
+        <v>244</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="7" t="s">
-        <v>168</v>
+        <v>131</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>169</v>
+        <v>245</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>170</v>
+        <v>246</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>171</v>
+        <v>247</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>172</v>
+        <v>248</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>173</v>
+        <v>249</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B3" s="8" t="n">
         <v>42</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>174</v>
+        <v>250</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>175</v>
+        <v>251</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>176</v>
+        <v>252</v>
       </c>
       <c r="F3" s="16" t="s">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>178</v>
+        <v>254</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>43</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>179</v>
+        <v>255</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>180</v>
+        <v>256</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>181</v>
+        <v>257</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>182</v>
+        <v>258</v>
       </c>
       <c r="G4" s="8" t="s">
-        <v>183</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>19</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>184</v>
+        <v>260</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>185</v>
+        <v>261</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>186</v>
+        <v>262</v>
       </c>
       <c r="F5" s="16" t="s">
-        <v>177</v>
+        <v>253</v>
       </c>
       <c r="G5" s="8" t="s">
-        <v>187</v>
+        <v>263</v>
       </c>
     </row>
   </sheetData>

</xml_diff>